<commit_message>
Build final delivery PDF with diagrams and updated cost estimates
Adds the exported Eraser diagrams, the PDF builder (adapted from the previous
delivery) and the rendered entrega.pdf. Cost workbooks rebuilt with the final
assumptions: on-demand only, everything as prod, 100 services at 2 vCPU/4 GB,
one peak month per year, 30 large single-AZ databases, c9g.large signers.
The two chosen cuts are backup-only DR and Service Connect instead of Lattice.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ATxWBSP6dN3Vdsj6c1eXyw
</commit_message>
<xml_diff>
--- a/docs/costos-actual.xlsx
+++ b/docs/costos-actual.xlsx
@@ -53,12 +53,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="4" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
@@ -426,15 +425,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F56"/>
+  <dimension ref="A1:F54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="66" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="58" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -535,34 +534,57 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="1" t="inlineStr">
-        <is>
-          <t>Cómputo (ECS en Fargate x86, sin Spot ni rightsizing)</t>
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>meses_pico</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Meses de pico al año (una semana, cuatro veces al año)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>meses</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Igual al objetivo (costos.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>tareas</t>
+          <t>mult_pico</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Tareas promedio de producción</t>
+          <t>Multiplicador de carga en pico</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
-        <v>200</v>
+        <v>3</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>tareas</t>
+          <t>x</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -574,25 +596,26 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>vcpu_tarea</t>
+          <t>factor</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>vCPU promedio por tarea</t>
-        </is>
-      </c>
-      <c r="C7" s="2" t="n">
-        <v>0.5</v>
+          <t>Factor de carga mensual promedio = (12 - meses de pico + meses de pico x multiplicador) / 12</t>
+        </is>
+      </c>
+      <c r="C7" s="2">
+        <f>(12-Supuestos!$C$5+Supuestos!$C$5*Supuestos!$C$6)/12</f>
+        <v/>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>vCPU</t>
+          <t>x</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
@@ -604,25 +627,25 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>gb_tarea</t>
+          <t>req_min</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Memoria promedio por tarea</t>
+          <t>Solicitudes por minuto (promedio fuera de pico)</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
-        <v>1</v>
+        <v>10000</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>req/min</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -634,147 +657,148 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>p_fg_vcpu</t>
+          <t>req_mes</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Fargate x86: precio por vCPU-hora</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="n">
-        <v>0.04048</v>
+          <t>Solicitudes por mes, con el factor de pico</t>
+        </is>
+      </c>
+      <c r="C9" s="2">
+        <f>Supuestos!$C$8*60*Supuestos!$C$3*Supuestos!$C$7</f>
+        <v/>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>solicitudes</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Verificar en calculadora</t>
+          <t>Calculado</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>p_fg_gb</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Fargate x86: precio por GB-hora</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="n">
-        <v>0.004445</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>Verificar en calculadora</t>
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Cómputo (ECS en Fargate x86, sin Graviton ni rightsizing)</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="1" t="inlineStr">
-        <is>
-          <t>Red</t>
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>servicios</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Servicios de ECS (una tarea equivalente por servicio)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>100</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>servicios</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Igual al objetivo (costos.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>alb_n</t>
+          <t>vcpu</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Número de ALB (varios clusters, sin consolidar)</t>
+          <t>vCPU promedio por servicio</t>
         </is>
       </c>
       <c r="C12" s="2" t="n">
-        <v>20</v>
+        <v>2</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>ALB</t>
+          <t>vCPU</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>3?</t>
+          <t>Igual al objetivo (costos.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>p_alb_h</t>
+          <t>gb</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>ALB: precio por hora</t>
-        </is>
-      </c>
-      <c r="C13" s="3" t="n">
-        <v>0.0225</v>
+          <t>Memoria promedio por servicio</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>4</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Verificar en calculadora</t>
+          <t>Igual al objetivo (costos.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>alb_lcu</t>
+          <t>p_fg_vcpu</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>LCU promedio por ALB</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="n">
-        <v>5</v>
+          <t>Fargate Linux x86: precio por vCPU-hora</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>0.04048</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>LCU</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -782,21 +806,25 @@
           <t>sí</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Verificar en calculadora</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>p_alb_lcu</t>
+          <t>p_fg_gb</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>ALB: precio por LCU-hora</t>
+          <t>Fargate Linux x86: precio por GB-hora</t>
         </is>
       </c>
       <c r="C15" s="3" t="n">
-        <v>0.008</v>
+        <v>0.004445</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
@@ -815,57 +843,34 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>req_min</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>Solicitudes por minuto</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="n">
-        <v>10000</v>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>req/min</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>no</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>Dato del escenario</t>
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>Red</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>waf_reglas</t>
+          <t>alb_n</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>WAF: reglas</t>
+          <t>ALB (uno por servicio)</t>
         </is>
       </c>
       <c r="C17" s="2" t="n">
-        <v>15</v>
+        <v>100</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>reglas</t>
+          <t>ALB</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -877,16 +882,16 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>p_waf_acl</t>
+          <t>p_alb_h</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>WAF: precio por web ACL al mes</t>
+          <t>ALB: precio por hora</t>
         </is>
       </c>
       <c r="C18" s="3" t="n">
-        <v>5</v>
+        <v>0.0225</v>
       </c>
       <c r="D18" t="inlineStr">
         <is>
@@ -907,20 +912,20 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>p_waf_regla</t>
+          <t>lcu</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>WAF: precio por regla al mes</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="n">
-        <v>1</v>
+          <t>LCU promedio total entre todos los ALB</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>50</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>LCU</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -930,23 +935,23 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Verificar en calculadora</t>
+          <t>Igual al objetivo (costos.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>p_waf_req</t>
+          <t>p_alb_lcu</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>WAF: precio por millón de solicitudes</t>
+          <t>ALB: precio por LCU-hora</t>
         </is>
       </c>
       <c r="C20" s="3" t="n">
-        <v>0.6</v>
+        <v>0.008</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
@@ -967,20 +972,20 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>nat_n</t>
+          <t>waf_reglas</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>NAT gateways</t>
+          <t>WAF: reglas</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>NAT</t>
+          <t>reglas</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -997,16 +1002,16 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>p_nat_h</t>
+          <t>p_waf_acl</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>NAT: precio por hora</t>
+          <t>WAF: precio por web ACL al mes</t>
         </is>
       </c>
       <c r="C22" s="3" t="n">
-        <v>0.045</v>
+        <v>5</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
@@ -1027,20 +1032,20 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>nat_gb</t>
+          <t>p_waf_regla</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>NAT: GB procesados por mes</t>
-        </is>
-      </c>
-      <c r="C23" s="2" t="n">
-        <v>3000</v>
+          <t>WAF: precio por regla al mes</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>1</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1050,23 +1055,23 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Igual al objetivo (costos.xlsx)</t>
+          <t>Verificar en calculadora</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>p_nat_gb</t>
+          <t>p_waf_req</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>NAT: precio por GB</t>
+          <t>WAF: precio por millón de solicitudes</t>
         </is>
       </c>
       <c r="C24" s="3" t="n">
-        <v>0.045</v>
+        <v>0.6</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
@@ -1087,20 +1092,20 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>vpn_n</t>
+          <t>nat_n</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>VPN: instancias de un appliance de terceros</t>
+          <t>NAT gateways</t>
         </is>
       </c>
       <c r="C25" s="2" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>instancias</t>
+          <t>NAT</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -1110,23 +1115,23 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>2? Producto y costo desconocidos</t>
+          <t>Igual al objetivo (costos.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>p_vpn</t>
+          <t>p_nat_h</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>VPN: precio por hora de la instancia (sin licencia)</t>
+          <t>NAT: precio por hora</t>
         </is>
       </c>
       <c r="C26" s="3" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.045</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
@@ -1140,34 +1145,57 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Ej. c6i.large; licencia excluida</t>
+          <t>Verificar en calculadora</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="1" t="inlineStr">
-        <is>
-          <t>Datos</t>
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>nat_gb</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>NAT: GB procesados por mes fuera de pico</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="n">
+        <v>3000</v>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>GB</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>sí</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>Igual al objetivo (costos.xlsx)</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>rds_g_n</t>
+          <t>p_nat_gb</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>RDS grandes (Multi-AZ)</t>
-        </is>
-      </c>
-      <c r="C28" s="2" t="n">
-        <v>5</v>
+          <t>NAT: precio por GB</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>0.045</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>instancias</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -1177,27 +1205,27 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Igual al objetivo (costos.xlsx)</t>
+          <t>Verificar en calculadora</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>p_rds_g</t>
+          <t>vpn_n</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>RDS grande x86 Multi-AZ: precio por hora</t>
-        </is>
-      </c>
-      <c r="C29" s="3" t="n">
+          <t>VPN de terceros: instancias del appliance</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="n">
         <v>1</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>USD</t>
+          <t>instancias</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -1207,27 +1235,27 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Ej. db.r6i.xlarge; depende del motor</t>
+          <t>2? Producto y costo desconocidos</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>rds_m_n</t>
+          <t>p_vpn</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>RDS medianas (Multi-AZ)</t>
-        </is>
-      </c>
-      <c r="C30" s="2" t="n">
-        <v>10</v>
+          <t>VPN: precio por hora de la instancia, sin licencia (ej. c6i.large)</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>0.08500000000000001</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>instancias</t>
+          <t>USD</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -1237,53 +1265,30 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Igual al objetivo (costos.xlsx)</t>
+          <t>Verificar en calculadora</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>p_rds_m</t>
-        </is>
-      </c>
-      <c r="B31" t="inlineStr">
-        <is>
-          <t>RDS mediana x86 Multi-AZ: precio por hora</t>
-        </is>
-      </c>
-      <c r="C31" s="3" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="D31" t="inlineStr">
-        <is>
-          <t>USD</t>
-        </is>
-      </c>
-      <c r="E31" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="F31" t="inlineStr">
-        <is>
-          <t>Ej. db.r6i.large; depende del motor</t>
+      <c r="A31" s="1" t="inlineStr">
+        <is>
+          <t>Datos</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>rds_p_n</t>
+          <t>rds_n</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>RDS pequeñas (Multi-AZ)</t>
+          <t>RDS PostgreSQL: instancias grandes en una zona</t>
         </is>
       </c>
       <c r="C32" s="2" t="n">
-        <v>15</v>
+        <v>30</v>
       </c>
       <c r="D32" t="inlineStr">
         <is>
@@ -1292,7 +1297,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -1304,16 +1309,16 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>p_rds_p</t>
+          <t>p_rds</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>RDS pequeña x86 Multi-AZ: precio por hora</t>
+          <t>RDS PostgreSQL db.r6i.xlarge Single-AZ: precio por hora</t>
         </is>
       </c>
       <c r="C33" s="3" t="n">
-        <v>0.136</v>
+        <v>0.5</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
@@ -1327,7 +1332,7 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Ej. db.t3.medium; depende del motor</t>
+          <t>Verificar en calculadora</t>
         </is>
       </c>
     </row>
@@ -1339,7 +1344,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Almacenamiento total RDS</t>
+          <t>RDS: almacenamiento total</t>
         </is>
       </c>
       <c r="C34" s="2" t="n">
@@ -1369,11 +1374,11 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Almacenamiento Multi-AZ: precio por GB-mes</t>
+          <t>RDS gp2 Single-AZ: precio por GB-mes</t>
         </is>
       </c>
       <c r="C35" s="3" t="n">
-        <v>0.23</v>
+        <v>0.115</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
@@ -1429,7 +1434,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>OpenSearch: precio por hora del nodo de datos</t>
+          <t>OpenSearch: precio por hora del nodo de datos (r6g.large.search)</t>
         </is>
       </c>
       <c r="C37" s="3" t="n">
@@ -1447,7 +1452,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Ej. r6g.large.search</t>
+          <t>Verificar en calculadora</t>
         </is>
       </c>
     </row>
@@ -1489,7 +1494,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>OpenSearch: precio por hora del nodo maestro</t>
+          <t>OpenSearch: precio por hora del nodo maestro (m6g.large.search)</t>
         </is>
       </c>
       <c r="C39" s="3" t="n">
@@ -1507,7 +1512,7 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Ej. m6g.large.search</t>
+          <t>Verificar en calculadora</t>
         </is>
       </c>
     </row>
@@ -1523,7 +1528,7 @@
         </is>
       </c>
       <c r="C40" s="2" t="n">
-        <v>1500</v>
+        <v>100</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
@@ -1532,12 +1537,12 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>500 GB x 3 nodos</t>
+          <t>S-05</t>
         </is>
       </c>
     </row>
@@ -1549,7 +1554,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>OpenSearch: precio por GB-mes de EBS</t>
+          <t>OpenSearch: precio por GB-mes de EBS gp3</t>
         </is>
       </c>
       <c r="C41" s="3" t="n">
@@ -1581,42 +1586,46 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>kms_llaves</t>
+          <t>firmas</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Llaves de KMS de uso general</t>
+          <t>Firmas por mes</t>
         </is>
       </c>
       <c r="C43" s="2" t="n">
-        <v>10</v>
+        <v>10000000</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>llaves</t>
+          <t>firmas</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="F43" t="inlineStr"/>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Igual al objetivo (costos.xlsx)</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>kms_wallets</t>
+          <t>kms_llaves</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Llaves de KMS adicionales, una por wallet</t>
+          <t>Llaves de KMS de uso general (las llaves de wallets están en RDS)</t>
         </is>
       </c>
       <c r="C44" s="2" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
@@ -1630,7 +1639,7 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>10? Si hoy hay una llave por wallet, poner el número de wallets</t>
+          <t>10?</t>
         </is>
       </c>
     </row>
@@ -1675,8 +1684,9 @@
           <t>KMS: solicitudes por mes</t>
         </is>
       </c>
-      <c r="C46" s="2" t="n">
-        <v>20000000</v>
+      <c r="C46" s="2">
+        <f>Supuestos!$C$43*2</f>
+        <v/>
       </c>
       <c r="D46" t="inlineStr">
         <is>
@@ -1685,7 +1695,7 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>sí</t>
+          <t>no</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
@@ -1702,7 +1712,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>KMS: precio por 10 mil solicitudes</t>
+          <t>KMS: precio por 10 mil solicitudes (sin capa gratuita)</t>
         </is>
       </c>
       <c r="C47" s="3" t="n">
@@ -1799,7 +1809,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>CloudWatch Logs: GB ingeridos por mes</t>
+          <t>CloudWatch Logs: GB ingeridos por mes fuera de pico</t>
         </is>
       </c>
       <c r="C51" s="2" t="n">
@@ -1908,43 +1918,6 @@
       <c r="F54" t="inlineStr">
         <is>
           <t>Verificar en calculadora</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" s="1" t="inlineStr">
-        <is>
-          <t>No productivo (en la misma cuenta)</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>np_pct</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>No productivo: proporción del cómputo y datos de producción</t>
-        </is>
-      </c>
-      <c r="C56" s="4" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>%</t>
-        </is>
-      </c>
-      <c r="E56" t="inlineStr">
-        <is>
-          <t>sí</t>
-        </is>
-      </c>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>Igual a staging + dev del objetivo, sin apagado fuera de horario</t>
         </is>
       </c>
     </row>
@@ -1959,16 +1932,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="50" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2021,11 +1996,11 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>vCPU-hora bajo demanda</t>
+          <t>vCPU-hora</t>
         </is>
       </c>
       <c r="D2" s="2">
-        <f>Supuestos!$C$6*Supuestos!$C$7*Supuestos!$C$3</f>
+        <f>Supuestos!$C$11*Supuestos!$C$12*Supuestos!$C$3*Supuestos!$C$7</f>
         <v/>
       </c>
       <c r="E2" t="inlineStr">
@@ -2034,10 +2009,10 @@
         </is>
       </c>
       <c r="F2" s="3">
-        <f>Supuestos!$C$9</f>
-        <v/>
-      </c>
-      <c r="G2" s="5">
+        <f>Supuestos!$C$14</f>
+        <v/>
+      </c>
+      <c r="G2" s="4">
         <f>D2*F2</f>
         <v/>
       </c>
@@ -2055,11 +2030,11 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>GB-hora bajo demanda</t>
+          <t>GB-hora</t>
         </is>
       </c>
       <c r="D3" s="2">
-        <f>Supuestos!$C$6*Supuestos!$C$8*Supuestos!$C$3</f>
+        <f>Supuestos!$C$11*Supuestos!$C$13*Supuestos!$C$3*Supuestos!$C$7</f>
         <v/>
       </c>
       <c r="E3" t="inlineStr">
@@ -2068,10 +2043,10 @@
         </is>
       </c>
       <c r="F3" s="3">
-        <f>Supuestos!$C$10</f>
-        <v/>
-      </c>
-      <c r="G3" s="5">
+        <f>Supuestos!$C$15</f>
+        <v/>
+      </c>
+      <c r="G3" s="4">
         <f>D3*F3</f>
         <v/>
       </c>
@@ -2093,7 +2068,7 @@
         </is>
       </c>
       <c r="D4" s="2">
-        <f>Supuestos!$C$12*Supuestos!$C$3</f>
+        <f>Supuestos!$C$17*Supuestos!$C$3</f>
         <v/>
       </c>
       <c r="E4" t="inlineStr">
@@ -2102,10 +2077,10 @@
         </is>
       </c>
       <c r="F4" s="3">
-        <f>Supuestos!$C$13</f>
-        <v/>
-      </c>
-      <c r="G4" s="5">
+        <f>Supuestos!$C$18</f>
+        <v/>
+      </c>
+      <c r="G4" s="4">
         <f>D4*F4</f>
         <v/>
       </c>
@@ -2127,7 +2102,7 @@
         </is>
       </c>
       <c r="D5" s="2">
-        <f>Supuestos!$C$12*Supuestos!$C$14*Supuestos!$C$3</f>
+        <f>Supuestos!$C$19*Supuestos!$C$3*Supuestos!$C$7</f>
         <v/>
       </c>
       <c r="E5" t="inlineStr">
@@ -2136,10 +2111,10 @@
         </is>
       </c>
       <c r="F5" s="3">
-        <f>Supuestos!$C$15</f>
-        <v/>
-      </c>
-      <c r="G5" s="5">
+        <f>Supuestos!$C$20</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
         <f>D5*F5</f>
         <v/>
       </c>
@@ -2170,10 +2145,10 @@
         </is>
       </c>
       <c r="F6" s="3">
-        <f>Supuestos!$C$18+Supuestos!$C$17*Supuestos!$C$19</f>
-        <v/>
-      </c>
-      <c r="G6" s="5">
+        <f>Supuestos!$C$22+Supuestos!$C$21*Supuestos!$C$23</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
         <f>D6*F6</f>
         <v/>
       </c>
@@ -2195,7 +2170,7 @@
         </is>
       </c>
       <c r="D7" s="2">
-        <f>(Supuestos!$C$16*60*Supuestos!$C$3)/1000000</f>
+        <f>Supuestos!$C$9/1000000</f>
         <v/>
       </c>
       <c r="E7" t="inlineStr">
@@ -2204,10 +2179,10 @@
         </is>
       </c>
       <c r="F7" s="3">
-        <f>Supuestos!$C$20</f>
-        <v/>
-      </c>
-      <c r="G7" s="5">
+        <f>Supuestos!$C$24</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
         <f>D7*F7</f>
         <v/>
       </c>
@@ -2229,7 +2204,7 @@
         </is>
       </c>
       <c r="D8" s="2">
-        <f>Supuestos!$C$21*Supuestos!$C$3</f>
+        <f>Supuestos!$C$25*Supuestos!$C$3</f>
         <v/>
       </c>
       <c r="E8" t="inlineStr">
@@ -2238,10 +2213,10 @@
         </is>
       </c>
       <c r="F8" s="3">
-        <f>Supuestos!$C$22</f>
-        <v/>
-      </c>
-      <c r="G8" s="5">
+        <f>Supuestos!$C$26</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
         <f>D8*F8</f>
         <v/>
       </c>
@@ -2263,7 +2238,7 @@
         </is>
       </c>
       <c r="D9" s="2">
-        <f>Supuestos!$C$23</f>
+        <f>Supuestos!$C$27*Supuestos!$C$7</f>
         <v/>
       </c>
       <c r="E9" t="inlineStr">
@@ -2272,10 +2247,10 @@
         </is>
       </c>
       <c r="F9" s="3">
-        <f>Supuestos!$C$24</f>
-        <v/>
-      </c>
-      <c r="G9" s="5">
+        <f>Supuestos!$C$28</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
         <f>D9*F9</f>
         <v/>
       </c>
@@ -2297,7 +2272,7 @@
         </is>
       </c>
       <c r="D10" s="2">
-        <f>Supuestos!$C$25*Supuestos!$C$3</f>
+        <f>Supuestos!$C$29*Supuestos!$C$3</f>
         <v/>
       </c>
       <c r="E10" t="inlineStr">
@@ -2306,10 +2281,10 @@
         </is>
       </c>
       <c r="F10" s="3">
-        <f>Supuestos!$C$26</f>
-        <v/>
-      </c>
-      <c r="G10" s="5">
+        <f>Supuestos!$C$30</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
         <f>D10*F10</f>
         <v/>
       </c>
@@ -2322,16 +2297,16 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>RDS</t>
+          <t>RDS PostgreSQL</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Instancias grandes Multi-AZ</t>
+          <t>Instancias grandes Single-AZ</t>
         </is>
       </c>
       <c r="D11" s="2">
-        <f>Supuestos!$C$28*Supuestos!$C$3</f>
+        <f>Supuestos!$C$32*Supuestos!$C$3</f>
         <v/>
       </c>
       <c r="E11" t="inlineStr">
@@ -2340,10 +2315,10 @@
         </is>
       </c>
       <c r="F11" s="3">
-        <f>Supuestos!$C$29</f>
-        <v/>
-      </c>
-      <c r="G11" s="5">
+        <f>Supuestos!$C$33</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
         <f>D11*F11</f>
         <v/>
       </c>
@@ -2356,28 +2331,28 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>RDS</t>
+          <t>RDS PostgreSQL</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Instancias medianas Multi-AZ</t>
+          <t>Almacenamiento</t>
         </is>
       </c>
       <c r="D12" s="2">
-        <f>Supuestos!$C$30*Supuestos!$C$3</f>
+        <f>Supuestos!$C$34</f>
         <v/>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>instancia-h</t>
+          <t>GB-mes</t>
         </is>
       </c>
       <c r="F12" s="3">
-        <f>Supuestos!$C$31</f>
-        <v/>
-      </c>
-      <c r="G12" s="5">
+        <f>Supuestos!$C$35</f>
+        <v/>
+      </c>
+      <c r="G12" s="4">
         <f>D12*F12</f>
         <v/>
       </c>
@@ -2390,28 +2365,28 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>RDS</t>
+          <t>OpenSearch (dominio)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Instancias pequeñas Multi-AZ</t>
+          <t>Nodos de datos</t>
         </is>
       </c>
       <c r="D13" s="2">
-        <f>Supuestos!$C$32*Supuestos!$C$3</f>
+        <f>Supuestos!$C$36*Supuestos!$C$3</f>
         <v/>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>instancia-h</t>
+          <t>nodo-h</t>
         </is>
       </c>
       <c r="F13" s="3">
-        <f>Supuestos!$C$33</f>
-        <v/>
-      </c>
-      <c r="G13" s="5">
+        <f>Supuestos!$C$37</f>
+        <v/>
+      </c>
+      <c r="G13" s="4">
         <f>D13*F13</f>
         <v/>
       </c>
@@ -2424,28 +2399,28 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>RDS</t>
+          <t>OpenSearch (dominio)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Almacenamiento</t>
+          <t>Nodos maestros</t>
         </is>
       </c>
       <c r="D14" s="2">
-        <f>Supuestos!$C$34</f>
+        <f>Supuestos!$C$38*Supuestos!$C$3</f>
         <v/>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>GB-mes</t>
+          <t>nodo-h</t>
         </is>
       </c>
       <c r="F14" s="3">
-        <f>Supuestos!$C$35</f>
-        <v/>
-      </c>
-      <c r="G14" s="5">
+        <f>Supuestos!$C$39</f>
+        <v/>
+      </c>
+      <c r="G14" s="4">
         <f>D14*F14</f>
         <v/>
       </c>
@@ -2463,23 +2438,23 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Nodos de datos</t>
+          <t>Almacenamiento EBS</t>
         </is>
       </c>
       <c r="D15" s="2">
-        <f>Supuestos!$C$36*Supuestos!$C$3</f>
+        <f>Supuestos!$C$40</f>
         <v/>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>nodo-h</t>
+          <t>GB-mes</t>
         </is>
       </c>
       <c r="F15" s="3">
-        <f>Supuestos!$C$37</f>
-        <v/>
-      </c>
-      <c r="G15" s="5">
+        <f>Supuestos!$C$41</f>
+        <v/>
+      </c>
+      <c r="G15" s="4">
         <f>D15*F15</f>
         <v/>
       </c>
@@ -2487,33 +2462,33 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Datos</t>
+          <t>Llaves y secretos</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>OpenSearch (dominio)</t>
+          <t>AWS KMS</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Nodos maestros</t>
+          <t>Llaves de uso general</t>
         </is>
       </c>
       <c r="D16" s="2">
-        <f>Supuestos!$C$38*Supuestos!$C$3</f>
+        <f>Supuestos!$C$44</f>
         <v/>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>nodo-h</t>
+          <t>llaves</t>
         </is>
       </c>
       <c r="F16" s="3">
-        <f>Supuestos!$C$39</f>
-        <v/>
-      </c>
-      <c r="G16" s="5">
+        <f>Supuestos!$C$45</f>
+        <v/>
+      </c>
+      <c r="G16" s="4">
         <f>D16*F16</f>
         <v/>
       </c>
@@ -2521,33 +2496,33 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Datos</t>
+          <t>Llaves y secretos</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>OpenSearch (dominio)</t>
+          <t>AWS KMS</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Almacenamiento EBS</t>
+          <t>Solicitudes</t>
         </is>
       </c>
       <c r="D17" s="2">
-        <f>Supuestos!$C$40</f>
+        <f>Supuestos!$C$46/10000</f>
         <v/>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>GB-mes</t>
+          <t>10 mil</t>
         </is>
       </c>
       <c r="F17" s="3">
-        <f>Supuestos!$C$41</f>
-        <v/>
-      </c>
-      <c r="G17" s="5">
+        <f>Supuestos!$C$47</f>
+        <v/>
+      </c>
+      <c r="G17" s="4">
         <f>D17*F17</f>
         <v/>
       </c>
@@ -2560,28 +2535,28 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AWS KMS</t>
+          <t>Secrets Manager</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Llaves de uso general y por wallet</t>
+          <t>Secretos</t>
         </is>
       </c>
       <c r="D18" s="2">
-        <f>Supuestos!$C$43+Supuestos!$C$44</f>
+        <f>Supuestos!$C$48</f>
         <v/>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>llaves</t>
+          <t>secretos</t>
         </is>
       </c>
       <c r="F18" s="3">
-        <f>Supuestos!$C$45</f>
-        <v/>
-      </c>
-      <c r="G18" s="5">
+        <f>Supuestos!$C$49</f>
+        <v/>
+      </c>
+      <c r="G18" s="4">
         <f>D18*F18</f>
         <v/>
       </c>
@@ -2589,33 +2564,33 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Llaves y secretos</t>
+          <t>Observabilidad</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>AWS KMS</t>
+          <t>CloudWatch Logs</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Solicitudes</t>
+          <t>Ingesta</t>
         </is>
       </c>
       <c r="D19" s="2">
-        <f>Supuestos!$C$46/10000</f>
+        <f>Supuestos!$C$51*Supuestos!$C$7</f>
         <v/>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>10 mil</t>
+          <t>GB</t>
         </is>
       </c>
       <c r="F19" s="3">
-        <f>Supuestos!$C$47</f>
-        <v/>
-      </c>
-      <c r="G19" s="5">
+        <f>Supuestos!$C$52</f>
+        <v/>
+      </c>
+      <c r="G19" s="4">
         <f>D19*F19</f>
         <v/>
       </c>
@@ -2623,33 +2598,33 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Llaves y secretos</t>
+          <t>Observabilidad</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Secrets Manager</t>
+          <t>CloudWatch Logs</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Secretos</t>
+          <t>Almacenamiento acumulado sin retención</t>
         </is>
       </c>
       <c r="D20" s="2">
-        <f>Supuestos!$C$48</f>
+        <f>Supuestos!$C$51*Supuestos!$C$7*Supuestos!$C$53</f>
         <v/>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>secretos</t>
+          <t>GB-mes</t>
         </is>
       </c>
       <c r="F20" s="3">
-        <f>Supuestos!$C$49</f>
-        <v/>
-      </c>
-      <c r="G20" s="5">
+        <f>Supuestos!$C$54</f>
+        <v/>
+      </c>
+      <c r="G20" s="4">
         <f>D20*F20</f>
         <v/>
       </c>
@@ -2657,33 +2632,33 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
+          <t>Gobierno</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CloudWatch Logs</t>
+          <t>AWS Config / Security Hub</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Ingesta</t>
+          <t>No existe hoy</t>
         </is>
       </c>
       <c r="D21" s="2">
-        <f>Supuestos!$C$51</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>GB</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F21" s="3">
-        <f>Supuestos!$C$52</f>
-        <v/>
-      </c>
-      <c r="G21" s="5">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="G21" s="4">
         <f>D21*F21</f>
         <v/>
       </c>
@@ -2691,33 +2666,33 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
+          <t>CI/CD</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>CloudWatch Logs</t>
+          <t>Pipelines</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Almacenamiento acumulado sin retención</t>
+          <t>No existen hoy: cambios a mano</t>
         </is>
       </c>
       <c r="D22" s="2">
-        <f>Supuestos!$C$51*Supuestos!$C$53</f>
+        <f>0</f>
         <v/>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>GB-mes</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F22" s="3">
-        <f>Supuestos!$C$54</f>
-        <v/>
-      </c>
-      <c r="G22" s="5">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="G22" s="4">
         <f>D22*F22</f>
         <v/>
       </c>
@@ -2725,12 +2700,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gobierno</t>
+          <t>DR</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>AWS Config / Security Hub</t>
+          <t>Segunda región</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2751,250 +2726,137 @@
         <f>0</f>
         <v/>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="4">
         <f>D23*F23</f>
         <v/>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>CI/CD</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>Pipelines</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>No existen hoy: cambios a mano</t>
-        </is>
-      </c>
-      <c r="D24" s="2">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F24" s="3">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="G24" s="5">
-        <f>D24*F24</f>
-        <v/>
-      </c>
-    </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>DR</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>Segunda región</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>No existe hoy</t>
-        </is>
-      </c>
-      <c r="D25" s="2">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F25" s="3">
-        <f>0</f>
-        <v/>
-      </c>
-      <c r="G25" s="5">
-        <f>D25*F25</f>
-        <v/>
+      <c r="A25" s="1" t="inlineStr">
+        <is>
+          <t>Resumen</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>USD / mes</t>
+        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>No productivo</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>Misma cuenta</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>Cómputo y datos no productivos, encendidos 24/7</t>
-        </is>
-      </c>
-      <c r="D26" s="2">
-        <f>1</f>
-        <v/>
-      </c>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>mes</t>
-        </is>
-      </c>
-      <c r="F26" s="3">
-        <f>(SUMIFS(G2:G25,A2:A25,"Cómputo")+SUMIFS(G2:G25,A2:A25,"Datos"))*Supuestos!$C$56</f>
-        <v/>
-      </c>
-      <c r="G26" s="5">
-        <f>D26*F26</f>
+          <t>Cómputo</t>
+        </is>
+      </c>
+      <c r="G26" s="4">
+        <f>SUMIFS(G2:G23,A2:A23,"Cómputo")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="G27" s="4">
+        <f>SUMIFS(G2:G23,A2:A23,"Red")</f>
         <v/>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="1" t="inlineStr">
-        <is>
-          <t>Resumen</t>
-        </is>
-      </c>
-      <c r="G28" t="inlineStr">
-        <is>
-          <t>USD / mes</t>
-        </is>
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Datos</t>
+        </is>
+      </c>
+      <c r="G28" s="4">
+        <f>SUMIFS(G2:G23,A2:A23,"Datos")</f>
+        <v/>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Cómputo</t>
-        </is>
-      </c>
-      <c r="G29" s="5">
-        <f>SUMIFS(G2:G26,A2:A26,"Cómputo")</f>
+          <t>Llaves y secretos</t>
+        </is>
+      </c>
+      <c r="G29" s="4">
+        <f>SUMIFS(G2:G23,A2:A23,"Llaves y secretos")</f>
         <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Red</t>
-        </is>
-      </c>
-      <c r="G30" s="5">
-        <f>SUMIFS(G2:G26,A2:A26,"Red")</f>
+          <t>Observabilidad</t>
+        </is>
+      </c>
+      <c r="G30" s="4">
+        <f>SUMIFS(G2:G23,A2:A23,"Observabilidad")</f>
         <v/>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Datos</t>
-        </is>
-      </c>
-      <c r="G31" s="5">
-        <f>SUMIFS(G2:G26,A2:A26,"Datos")</f>
+          <t>Gobierno</t>
+        </is>
+      </c>
+      <c r="G31" s="4">
+        <f>SUMIFS(G2:G23,A2:A23,"Gobierno")</f>
         <v/>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Llaves y secretos</t>
-        </is>
-      </c>
-      <c r="G32" s="5">
-        <f>SUMIFS(G2:G26,A2:A26,"Llaves y secretos")</f>
+          <t>CI/CD</t>
+        </is>
+      </c>
+      <c r="G32" s="4">
+        <f>SUMIFS(G2:G23,A2:A23,"CI/CD")</f>
         <v/>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Observabilidad</t>
-        </is>
-      </c>
-      <c r="G33" s="5">
-        <f>SUMIFS(G2:G26,A2:A26,"Observabilidad")</f>
+          <t>DR</t>
+        </is>
+      </c>
+      <c r="G33" s="4">
+        <f>SUMIFS(G2:G23,A2:A23,"DR")</f>
         <v/>
       </c>
     </row>
     <row r="34">
-      <c r="A34" t="inlineStr">
-        <is>
-          <t>Gobierno</t>
+      <c r="A34" s="1" t="inlineStr">
+        <is>
+          <t>Total mensual</t>
         </is>
       </c>
       <c r="G34" s="5">
-        <f>SUMIFS(G2:G26,A2:A26,"Gobierno")</f>
+        <f>SUM(G2:G23)</f>
         <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>CI/CD</t>
-        </is>
-      </c>
-      <c r="G35" s="5">
-        <f>SUMIFS(G2:G26,A2:A26,"CI/CD")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" t="inlineStr">
-        <is>
-          <t>DR</t>
-        </is>
-      </c>
-      <c r="G36" s="5">
-        <f>SUMIFS(G2:G26,A2:A26,"DR")</f>
+          <t>Total anual</t>
+        </is>
+      </c>
+      <c r="G35" s="4">
+        <f>G34*12</f>
         <v/>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>No productivo</t>
-        </is>
-      </c>
-      <c r="G37" s="5">
-        <f>SUMIFS(G2:G26,A2:A26,"No productivo")</f>
-        <v/>
-      </c>
-    </row>
-    <row r="38">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>Total mensual</t>
-        </is>
-      </c>
-      <c r="G38" s="6">
-        <f>SUM(G2:G26)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="39">
-      <c r="A39" t="inlineStr">
-        <is>
-          <t>Total anual</t>
-        </is>
-      </c>
-      <c r="G39" s="5">
-        <f>G38*12</f>
-        <v/>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>Excluido: licencias de New Relic y de la VPN, plan de soporte de AWS, impuestos y costo del equipo.</t>
+          <t>Bajo demanda, sin capa gratuita, todo como producción. Excluido: licencias de New Relic y de la VPN, plan de soporte de AWS, impuestos y costo del equipo.</t>
         </is>
       </c>
     </row>

</xml_diff>